<commit_message>
Remove suspectEntity constraint for adverse event profile
Removed constraint on suspectEntity from IG Document Core. a322e6b5143ac5ee3adc38ceef3d202c96da2b09
</commit_message>
<xml_diff>
--- a/nr-doc-core-adverse-event/ig/StructureDefinition-extension-AdverseEvent.code.xlsx
+++ b/nr-doc-core-adverse-event/ig/StructureDefinition-extension-AdverseEvent.code.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-30T14:49:16+00:00</t>
+    <t>2026-09-16T12:34:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -347,7 +347,7 @@
     <t>required</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-origine-effet-indesirable-cisis|20260619134042</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-origine-effet-indesirable-cisis|20260716085851</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}

</xml_diff>